<commit_message>
Fonti del giorno dell'asta, e un altro refuso che rubava il rientro
Listone del 10 settembre: 595 righe, 532 in lista (P 63, D 190, C 193,
A 86), 63 fuori lista. Riallineati i conteggi fissi nei test.

Fasce, specialisti e calendario sono identici all'8 settembre: cambia
solo la data di scarico. Gli indisponibili no, passano da 58 a 60 voci.

Su Felici la fonte scrive "in dubbio per 29a" senza l'articolo, e
readMatchday() pretendeva "per la": una rottura del crociato finiva nel
dataset con matchday null, chip muto e nessun test rosso. Dopo il punto
di troppo su Piotrowski e' la seconda volta di fila, quindi adesso
articolo e punto sono entrambi opzionali.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015kvaptQA9vqY6jgfmisiPo
</commit_message>
<xml_diff>
--- a/data/lista_calciatori_classic.xlsx
+++ b/data/lista_calciatori_classic.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N595"/>
+  <dimension ref="A1:N596"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -2688,7 +2688,7 @@
         <v>5.83</v>
       </c>
       <c r="J60" s="2">
-        <v>6.67</v>
+        <v>6.83</v>
       </c>
       <c r="K60" s="2">
         <v>40</v>
@@ -20407,25 +20407,25 @@
     </row>
     <row r="527">
       <c r="A527" s="2">
-        <v>7628</v>
+        <v>7629</v>
       </c>
       <c r="B527" s="2" t="str">
-        <v>Sierro</v>
+        <v>Libra</v>
       </c>
       <c r="C527" s="2" t="str">
         <v/>
       </c>
       <c r="D527" s="2" t="str">
-        <v>Parma</v>
+        <v>Bologna</v>
       </c>
       <c r="E527" s="2">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F527" s="2" t="str">
         <v>C</v>
       </c>
       <c r="G527" s="2" t="str">
-        <v>M/C</v>
+        <v>C/T</v>
       </c>
       <c r="H527" s="2">
         <v>0</v>
@@ -20445,19 +20445,19 @@
     </row>
     <row r="528">
       <c r="A528" s="2">
-        <v>7572</v>
+        <v>7628</v>
       </c>
       <c r="B528" s="2" t="str">
-        <v>Comotto</v>
+        <v>Sierro</v>
       </c>
       <c r="C528" s="2" t="str">
         <v/>
       </c>
       <c r="D528" s="2" t="str">
-        <v>Milan</v>
+        <v>Parma</v>
       </c>
       <c r="E528" s="2">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F528" s="2" t="str">
         <v>C</v>
@@ -20483,25 +20483,25 @@
     </row>
     <row r="529">
       <c r="A529" s="2">
-        <v>7571</v>
+        <v>7572</v>
       </c>
       <c r="B529" s="2" t="str">
-        <v>Laerke</v>
+        <v>Comotto</v>
       </c>
       <c r="C529" s="2" t="str">
         <v/>
       </c>
       <c r="D529" s="2" t="str">
-        <v>Lecce</v>
+        <v>Milan</v>
       </c>
       <c r="E529" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F529" s="2" t="str">
         <v>C</v>
       </c>
       <c r="G529" s="2" t="str">
-        <v>W/A</v>
+        <v>M/C</v>
       </c>
       <c r="H529" s="2">
         <v>0</v>
@@ -20521,34 +20521,34 @@
     </row>
     <row r="530">
       <c r="A530" s="2">
-        <v>7481</v>
+        <v>7571</v>
       </c>
       <c r="B530" s="2" t="str">
-        <v>Dagasso</v>
+        <v>Laerke</v>
       </c>
       <c r="C530" s="2" t="str">
         <v/>
       </c>
       <c r="D530" s="2" t="str">
-        <v>Venezia</v>
+        <v>Lecce</v>
       </c>
       <c r="E530" s="2">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F530" s="2" t="str">
         <v>C</v>
       </c>
       <c r="G530" s="2" t="str">
-        <v>C</v>
+        <v>W/A</v>
       </c>
       <c r="H530" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I530" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J530" s="2">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="K530" s="2">
         <v>1</v>
@@ -20559,34 +20559,34 @@
     </row>
     <row r="531">
       <c r="A531" s="2">
-        <v>7456</v>
+        <v>7481</v>
       </c>
       <c r="B531" s="2" t="str">
-        <v>El Azzouzi A.</v>
+        <v>Dagasso</v>
       </c>
       <c r="C531" s="2" t="str">
         <v/>
       </c>
       <c r="D531" s="2" t="str">
-        <v>Frosinone</v>
+        <v>Venezia</v>
       </c>
       <c r="E531" s="2">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F531" s="2" t="str">
         <v>C</v>
       </c>
       <c r="G531" s="2" t="str">
-        <v>M/C</v>
+        <v>C</v>
       </c>
       <c r="H531" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I531" s="2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J531" s="2">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="K531" s="2">
         <v>1</v>
@@ -20597,25 +20597,25 @@
     </row>
     <row r="532">
       <c r="A532" s="2">
-        <v>7357</v>
+        <v>7456</v>
       </c>
       <c r="B532" s="2" t="str">
-        <v>Lahdo</v>
+        <v>El Azzouzi A.</v>
       </c>
       <c r="C532" s="2" t="str">
         <v/>
       </c>
       <c r="D532" s="2" t="str">
-        <v>Como</v>
+        <v>Frosinone</v>
       </c>
       <c r="E532" s="2">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F532" s="2" t="str">
         <v>C</v>
       </c>
       <c r="G532" s="2" t="str">
-        <v>C/T</v>
+        <v>M/C</v>
       </c>
       <c r="H532" s="2">
         <v>0</v>
@@ -20635,25 +20635,25 @@
     </row>
     <row r="533">
       <c r="A533" s="2">
-        <v>7319</v>
+        <v>7357</v>
       </c>
       <c r="B533" s="2" t="str">
-        <v>Fofana Sa.</v>
+        <v>Lahdo</v>
       </c>
       <c r="C533" s="2" t="str">
         <v/>
       </c>
       <c r="D533" s="2" t="str">
-        <v>Lecce</v>
+        <v>Como</v>
       </c>
       <c r="E533" s="2">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F533" s="2" t="str">
         <v>C</v>
       </c>
       <c r="G533" s="2" t="str">
-        <v>M/C</v>
+        <v>C/T</v>
       </c>
       <c r="H533" s="2">
         <v>0</v>
@@ -20673,19 +20673,19 @@
     </row>
     <row r="534">
       <c r="A534" s="2">
-        <v>7165</v>
+        <v>7319</v>
       </c>
       <c r="B534" s="2" t="str">
-        <v>Liteta</v>
+        <v>Fofana Sa.</v>
       </c>
       <c r="C534" s="2" t="str">
         <v/>
       </c>
       <c r="D534" s="2" t="str">
-        <v>Cagliari</v>
+        <v>Lecce</v>
       </c>
       <c r="E534" s="2">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F534" s="2" t="str">
         <v>C</v>
@@ -20711,19 +20711,19 @@
     </row>
     <row r="535">
       <c r="A535" s="2">
-        <v>7157</v>
+        <v>7165</v>
       </c>
       <c r="B535" s="2" t="str">
-        <v>Iannoni</v>
+        <v>Liteta</v>
       </c>
       <c r="C535" s="2" t="str">
-        <v>*</v>
+        <v/>
       </c>
       <c r="D535" s="2" t="str">
-        <v>Sassuolo</v>
+        <v>Cagliari</v>
       </c>
       <c r="E535" s="2">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F535" s="2" t="str">
         <v>C</v>
@@ -20749,177 +20749,177 @@
     </row>
     <row r="536">
       <c r="A536" s="2">
-        <v>6592</v>
+        <v>7157</v>
       </c>
       <c r="B536" s="2" t="str">
-        <v>Forson O.</v>
+        <v>Iannoni</v>
       </c>
       <c r="C536" s="2" t="str">
-        <v/>
+        <v>*</v>
       </c>
       <c r="D536" s="2" t="str">
-        <v>Monza</v>
+        <v>Sassuolo</v>
       </c>
       <c r="E536" s="2">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F536" s="2" t="str">
         <v>C</v>
       </c>
       <c r="G536" s="2" t="str">
-        <v>W/T</v>
+        <v>M/C</v>
       </c>
       <c r="H536" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I536" s="2">
-        <v>5.75</v>
+        <v>0</v>
       </c>
       <c r="J536" s="2">
-        <v>5.75</v>
+        <v>0</v>
       </c>
       <c r="K536" s="2">
         <v>1</v>
       </c>
       <c r="L536" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2">
-        <v>5462</v>
+        <v>6592</v>
       </c>
       <c r="B537" s="2" t="str">
-        <v>Ciervo</v>
+        <v>Forson O.</v>
       </c>
       <c r="C537" s="2" t="str">
         <v/>
       </c>
       <c r="D537" s="2" t="str">
-        <v>Cagliari</v>
+        <v>Monza</v>
       </c>
       <c r="E537" s="2">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F537" s="2" t="str">
         <v>C</v>
       </c>
       <c r="G537" s="2" t="str">
-        <v>W</v>
+        <v>W/T</v>
       </c>
       <c r="H537" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I537" s="2">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="J537" s="2">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="K537" s="2">
         <v>1</v>
       </c>
       <c r="L537" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2">
-        <v>7615</v>
+        <v>5462</v>
       </c>
       <c r="B538" s="2" t="str">
-        <v>Drobnic</v>
+        <v>Ciervo</v>
       </c>
       <c r="C538" s="2" t="str">
         <v/>
       </c>
       <c r="D538" s="2" t="str">
-        <v>Parma</v>
+        <v>Cagliari</v>
       </c>
       <c r="E538" s="2">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F538" s="2" t="str">
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="G538" s="2" t="str">
-        <v>Dc</v>
+        <v>W</v>
       </c>
       <c r="H538" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I538" s="2">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="J538" s="2">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="K538" s="2">
         <v>1</v>
       </c>
       <c r="L538" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2">
-        <v>7604</v>
+        <v>7615</v>
       </c>
       <c r="B539" s="2" t="str">
-        <v>Maye</v>
+        <v>Drobnic</v>
       </c>
       <c r="C539" s="2" t="str">
         <v/>
       </c>
       <c r="D539" s="2" t="str">
-        <v>Monza</v>
+        <v>Parma</v>
       </c>
       <c r="E539" s="2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F539" s="2" t="str">
         <v>D</v>
       </c>
       <c r="G539" s="2" t="str">
-        <v>Ds/Dc</v>
+        <v>Dc</v>
       </c>
       <c r="H539" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I539" s="2">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="J539" s="2">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="K539" s="2">
         <v>1</v>
       </c>
       <c r="L539" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2">
-        <v>7553</v>
+        <v>7604</v>
       </c>
       <c r="B540" s="2" t="str">
-        <v>Omar Fayed</v>
+        <v>Maye</v>
       </c>
       <c r="C540" s="2" t="str">
         <v/>
       </c>
       <c r="D540" s="2" t="str">
-        <v>Frosinone</v>
+        <v>Monza</v>
       </c>
       <c r="E540" s="2">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F540" s="2" t="str">
         <v>D</v>
       </c>
       <c r="G540" s="2" t="str">
-        <v>Dc</v>
+        <v>Ds/Dc</v>
       </c>
       <c r="H540" s="2">
         <v>0</v>
@@ -20939,25 +20939,25 @@
     </row>
     <row r="541">
       <c r="A541" s="2">
-        <v>7471</v>
+        <v>7553</v>
       </c>
       <c r="B541" s="2" t="str">
-        <v>Corrado</v>
+        <v>Omar Fayed</v>
       </c>
       <c r="C541" s="2" t="str">
-        <v>*</v>
+        <v/>
       </c>
       <c r="D541" s="2" t="str">
         <v>Frosinone</v>
       </c>
       <c r="E541" s="2">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F541" s="2" t="str">
         <v>D</v>
       </c>
       <c r="G541" s="2" t="str">
-        <v>Ds/E</v>
+        <v>Dc</v>
       </c>
       <c r="H541" s="2">
         <v>0</v>
@@ -20977,10 +20977,10 @@
     </row>
     <row r="542">
       <c r="A542" s="2">
-        <v>7468</v>
+        <v>7471</v>
       </c>
       <c r="B542" s="2" t="str">
-        <v>Gelli J.</v>
+        <v>Corrado</v>
       </c>
       <c r="C542" s="2" t="str">
         <v>*</v>
@@ -20989,13 +20989,13 @@
         <v>Frosinone</v>
       </c>
       <c r="E542" s="2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F542" s="2" t="str">
         <v>D</v>
       </c>
       <c r="G542" s="2" t="str">
-        <v>Dc</v>
+        <v>Ds/E</v>
       </c>
       <c r="H542" s="2">
         <v>0</v>
@@ -21015,25 +21015,25 @@
     </row>
     <row r="543">
       <c r="A543" s="2">
-        <v>7454</v>
+        <v>7468</v>
       </c>
       <c r="B543" s="2" t="str">
-        <v>Gomes</v>
+        <v>Gelli J.</v>
       </c>
       <c r="C543" s="2" t="str">
-        <v/>
+        <v>*</v>
       </c>
       <c r="D543" s="2" t="str">
-        <v>Venezia</v>
+        <v>Frosinone</v>
       </c>
       <c r="E543" s="2">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F543" s="2" t="str">
         <v>D</v>
       </c>
       <c r="G543" s="2" t="str">
-        <v>Ds/Dc</v>
+        <v>Dc</v>
       </c>
       <c r="H543" s="2">
         <v>0</v>
@@ -21053,25 +21053,25 @@
     </row>
     <row r="544">
       <c r="A544" s="2">
-        <v>7396</v>
+        <v>7454</v>
       </c>
       <c r="B544" s="2" t="str">
-        <v>Macchioni</v>
+        <v>Gomes</v>
       </c>
       <c r="C544" s="2" t="str">
-        <v>*</v>
+        <v/>
       </c>
       <c r="D544" s="2" t="str">
-        <v>Sassuolo</v>
+        <v>Venezia</v>
       </c>
       <c r="E544" s="2">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F544" s="2" t="str">
         <v>D</v>
       </c>
       <c r="G544" s="2" t="str">
-        <v>Dc</v>
+        <v>Ds/Dc</v>
       </c>
       <c r="H544" s="2">
         <v>0</v>
@@ -21091,16 +21091,16 @@
     </row>
     <row r="545">
       <c r="A545" s="2">
-        <v>7346</v>
+        <v>7396</v>
       </c>
       <c r="B545" s="2" t="str">
-        <v>Raterink</v>
+        <v>Macchioni</v>
       </c>
       <c r="C545" s="2" t="str">
         <v>*</v>
       </c>
       <c r="D545" s="2" t="str">
-        <v>Cagliari</v>
+        <v>Sassuolo</v>
       </c>
       <c r="E545" s="2">
         <v>20</v>
@@ -21109,7 +21109,7 @@
         <v>D</v>
       </c>
       <c r="G545" s="2" t="str">
-        <v>Dd/E</v>
+        <v>Dc</v>
       </c>
       <c r="H545" s="2">
         <v>0</v>
@@ -21129,25 +21129,25 @@
     </row>
     <row r="546">
       <c r="A546" s="2">
-        <v>7164</v>
+        <v>7346</v>
       </c>
       <c r="B546" s="2" t="str">
-        <v>Perez M.</v>
+        <v>Raterink</v>
       </c>
       <c r="C546" s="2" t="str">
         <v>*</v>
       </c>
       <c r="D546" s="2" t="str">
-        <v>Lecce</v>
+        <v>Cagliari</v>
       </c>
       <c r="E546" s="2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F546" s="2" t="str">
         <v>D</v>
       </c>
       <c r="G546" s="2" t="str">
-        <v>Dd/Dc</v>
+        <v>Dd/E</v>
       </c>
       <c r="H546" s="2">
         <v>0</v>
@@ -21167,25 +21167,25 @@
     </row>
     <row r="547">
       <c r="A547" s="2">
-        <v>7156</v>
+        <v>7164</v>
       </c>
       <c r="B547" s="2" t="str">
-        <v>Pieragnolo</v>
+        <v>Perez M.</v>
       </c>
       <c r="C547" s="2" t="str">
-        <v/>
+        <v>*</v>
       </c>
       <c r="D547" s="2" t="str">
-        <v>Sassuolo</v>
+        <v>Lecce</v>
       </c>
       <c r="E547" s="2">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F547" s="2" t="str">
         <v>D</v>
       </c>
       <c r="G547" s="2" t="str">
-        <v>Ds/E</v>
+        <v>Dd/Dc</v>
       </c>
       <c r="H547" s="2">
         <v>0</v>
@@ -21205,25 +21205,25 @@
     </row>
     <row r="548">
       <c r="A548" s="2">
-        <v>5424</v>
+        <v>7156</v>
       </c>
       <c r="B548" s="2" t="str">
-        <v>Amey</v>
+        <v>Pieragnolo</v>
       </c>
       <c r="C548" s="2" t="str">
         <v/>
       </c>
       <c r="D548" s="2" t="str">
-        <v>Frosinone</v>
+        <v>Sassuolo</v>
       </c>
       <c r="E548" s="2">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F548" s="2" t="str">
         <v>D</v>
       </c>
       <c r="G548" s="2" t="str">
-        <v>Dc</v>
+        <v>Ds/E</v>
       </c>
       <c r="H548" s="2">
         <v>0</v>
@@ -21243,19 +21243,19 @@
     </row>
     <row r="549">
       <c r="A549" s="2">
-        <v>418</v>
+        <v>5424</v>
       </c>
       <c r="B549" s="2" t="str">
-        <v>Goldaniga</v>
+        <v>Amey</v>
       </c>
       <c r="C549" s="2" t="str">
         <v/>
       </c>
       <c r="D549" s="2" t="str">
-        <v>Como</v>
+        <v>Frosinone</v>
       </c>
       <c r="E549" s="2">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="F549" s="2" t="str">
         <v>D</v>
@@ -21281,16 +21281,16 @@
     </row>
     <row r="550">
       <c r="A550" s="2">
-        <v>327</v>
+        <v>418</v>
       </c>
       <c r="B550" s="2" t="str">
-        <v>Patric</v>
+        <v>Goldaniga</v>
       </c>
       <c r="C550" s="2" t="str">
         <v/>
       </c>
       <c r="D550" s="2" t="str">
-        <v>Lazio</v>
+        <v>Como</v>
       </c>
       <c r="E550" s="2">
         <v>33</v>
@@ -21299,7 +21299,7 @@
         <v>D</v>
       </c>
       <c r="G550" s="2" t="str">
-        <v>Dd/Dc</v>
+        <v>Dc</v>
       </c>
       <c r="H550" s="2">
         <v>0</v>
@@ -21319,25 +21319,25 @@
     </row>
     <row r="551">
       <c r="A551" s="2">
-        <v>7626</v>
+        <v>327</v>
       </c>
       <c r="B551" s="2" t="str">
-        <v>Pompei</v>
+        <v>Patric</v>
       </c>
       <c r="C551" s="2" t="str">
         <v/>
       </c>
       <c r="D551" s="2" t="str">
-        <v>Atalanta</v>
+        <v>Lazio</v>
       </c>
       <c r="E551" s="2">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="F551" s="2" t="str">
-        <v>P</v>
+        <v>D</v>
       </c>
       <c r="G551" s="2" t="str">
-        <v>Por</v>
+        <v>Dd/Dc</v>
       </c>
       <c r="H551" s="2">
         <v>0</v>
@@ -21357,19 +21357,19 @@
     </row>
     <row r="552">
       <c r="A552" s="2">
-        <v>7611</v>
+        <v>7626</v>
       </c>
       <c r="B552" s="2" t="str">
-        <v>Mrozek</v>
+        <v>Pompei</v>
       </c>
       <c r="C552" s="2" t="str">
         <v/>
       </c>
       <c r="D552" s="2" t="str">
-        <v>Udinese</v>
+        <v>Atalanta</v>
       </c>
       <c r="E552" s="2">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F552" s="2" t="str">
         <v>P</v>
@@ -21395,19 +21395,19 @@
     </row>
     <row r="553">
       <c r="A553" s="2">
-        <v>7603</v>
+        <v>7611</v>
       </c>
       <c r="B553" s="2" t="str">
-        <v>Grabara</v>
+        <v>Mrozek</v>
       </c>
       <c r="C553" s="2" t="str">
         <v/>
       </c>
       <c r="D553" s="2" t="str">
-        <v>Juventus</v>
+        <v>Udinese</v>
       </c>
       <c r="E553" s="2">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F553" s="2" t="str">
         <v>P</v>
@@ -21433,19 +21433,19 @@
     </row>
     <row r="554">
       <c r="A554" s="2">
-        <v>7560</v>
+        <v>7603</v>
       </c>
       <c r="B554" s="2" t="str">
-        <v>Pisseri</v>
+        <v>Grabara</v>
       </c>
       <c r="C554" s="2" t="str">
         <v/>
       </c>
       <c r="D554" s="2" t="str">
-        <v>Frosinone</v>
+        <v>Juventus</v>
       </c>
       <c r="E554" s="2">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="F554" s="2" t="str">
         <v>P</v>
@@ -21471,19 +21471,19 @@
     </row>
     <row r="555">
       <c r="A555" s="2">
-        <v>7557</v>
+        <v>7560</v>
       </c>
       <c r="B555" s="2" t="str">
-        <v>Penev</v>
+        <v>Pisseri</v>
       </c>
       <c r="C555" s="2" t="str">
         <v/>
       </c>
       <c r="D555" s="2" t="str">
-        <v>Lecce</v>
+        <v>Frosinone</v>
       </c>
       <c r="E555" s="2">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F555" s="2" t="str">
         <v>P</v>
@@ -21509,19 +21509,19 @@
     </row>
     <row r="556">
       <c r="A556" s="2">
-        <v>7545</v>
+        <v>7557</v>
       </c>
       <c r="B556" s="2" t="str">
-        <v>Vismara</v>
+        <v>Penev</v>
       </c>
       <c r="C556" s="2" t="str">
-        <v>*</v>
+        <v/>
       </c>
       <c r="D556" s="2" t="str">
-        <v>Atalanta</v>
+        <v>Lecce</v>
       </c>
       <c r="E556" s="2">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F556" s="2" t="str">
         <v>P</v>
@@ -21547,19 +21547,19 @@
     </row>
     <row r="557">
       <c r="A557" s="2">
-        <v>7534</v>
+        <v>7545</v>
       </c>
       <c r="B557" s="2" t="str">
-        <v>Renzetti</v>
+        <v>Vismara</v>
       </c>
       <c r="C557" s="2" t="str">
-        <v/>
+        <v>*</v>
       </c>
       <c r="D557" s="2" t="str">
-        <v>Lazio</v>
+        <v>Atalanta</v>
       </c>
       <c r="E557" s="2">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F557" s="2" t="str">
         <v>P</v>
@@ -21585,19 +21585,19 @@
     </row>
     <row r="558">
       <c r="A558" s="2">
-        <v>7533</v>
+        <v>7534</v>
       </c>
       <c r="B558" s="2" t="str">
-        <v>Happonen</v>
+        <v>Renzetti</v>
       </c>
       <c r="C558" s="2" t="str">
         <v/>
       </c>
       <c r="D558" s="2" t="str">
-        <v>Bologna</v>
+        <v>Lazio</v>
       </c>
       <c r="E558" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F558" s="2" t="str">
         <v>P</v>
@@ -21623,19 +21623,19 @@
     </row>
     <row r="559">
       <c r="A559" s="2">
-        <v>7531</v>
+        <v>7533</v>
       </c>
       <c r="B559" s="2" t="str">
-        <v>Pozzi</v>
+        <v>Happonen</v>
       </c>
       <c r="C559" s="2" t="str">
         <v/>
       </c>
       <c r="D559" s="2" t="str">
-        <v>Venezia</v>
+        <v>Bologna</v>
       </c>
       <c r="E559" s="2">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F559" s="2" t="str">
         <v>P</v>
@@ -21661,19 +21661,19 @@
     </row>
     <row r="560">
       <c r="A560" s="2">
-        <v>7475</v>
+        <v>7531</v>
       </c>
       <c r="B560" s="2" t="str">
-        <v>Strajnar</v>
+        <v>Pozzi</v>
       </c>
       <c r="C560" s="2" t="str">
         <v/>
       </c>
       <c r="D560" s="2" t="str">
-        <v>Monza</v>
+        <v>Venezia</v>
       </c>
       <c r="E560" s="2">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F560" s="2" t="str">
         <v>P</v>
@@ -21699,19 +21699,19 @@
     </row>
     <row r="561">
       <c r="A561" s="2">
-        <v>7466</v>
+        <v>7475</v>
       </c>
       <c r="B561" s="2" t="str">
-        <v>Lolic</v>
+        <v>Strajnar</v>
       </c>
       <c r="C561" s="2" t="str">
         <v/>
       </c>
       <c r="D561" s="2" t="str">
-        <v>Frosinone</v>
+        <v>Monza</v>
       </c>
       <c r="E561" s="2">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F561" s="2" t="str">
         <v>P</v>
@@ -21737,10 +21737,10 @@
     </row>
     <row r="562">
       <c r="A562" s="2">
-        <v>7463</v>
+        <v>7466</v>
       </c>
       <c r="B562" s="2" t="str">
-        <v>Desplanches</v>
+        <v>Lolic</v>
       </c>
       <c r="C562" s="2" t="str">
         <v/>
@@ -21749,7 +21749,7 @@
         <v>Frosinone</v>
       </c>
       <c r="E562" s="2">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F562" s="2" t="str">
         <v>P</v>
@@ -21775,19 +21775,19 @@
     </row>
     <row r="563">
       <c r="A563" s="2">
-        <v>7363</v>
+        <v>7463</v>
       </c>
       <c r="B563" s="2" t="str">
-        <v>Siviero</v>
+        <v>Desplanches</v>
       </c>
       <c r="C563" s="2" t="str">
         <v/>
       </c>
       <c r="D563" s="2" t="str">
-        <v>Torino</v>
+        <v>Frosinone</v>
       </c>
       <c r="E563" s="2">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F563" s="2" t="str">
         <v>P</v>
@@ -21813,19 +21813,19 @@
     </row>
     <row r="564">
       <c r="A564" s="2">
-        <v>7337</v>
+        <v>7363</v>
       </c>
       <c r="B564" s="2" t="str">
-        <v>Motta</v>
+        <v>Siviero</v>
       </c>
       <c r="C564" s="2" t="str">
         <v/>
       </c>
       <c r="D564" s="2" t="str">
-        <v>Lazio</v>
+        <v>Torino</v>
       </c>
       <c r="E564" s="2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F564" s="2" t="str">
         <v>P</v>
@@ -21851,19 +21851,19 @@
     </row>
     <row r="565">
       <c r="A565" s="2">
-        <v>7172</v>
+        <v>7337</v>
       </c>
       <c r="B565" s="2" t="str">
-        <v>Pessina Mas.</v>
+        <v>Motta</v>
       </c>
       <c r="C565" s="2" t="str">
         <v/>
       </c>
       <c r="D565" s="2" t="str">
-        <v>Bologna</v>
+        <v>Lazio</v>
       </c>
       <c r="E565" s="2">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F565" s="2" t="str">
         <v>P</v>
@@ -21889,16 +21889,16 @@
     </row>
     <row r="566">
       <c r="A566" s="2">
-        <v>7048</v>
+        <v>7172</v>
       </c>
       <c r="B566" s="2" t="str">
-        <v>De Marzi</v>
+        <v>Pessina Mas.</v>
       </c>
       <c r="C566" s="2" t="str">
         <v/>
       </c>
       <c r="D566" s="2" t="str">
-        <v>Roma</v>
+        <v>Bologna</v>
       </c>
       <c r="E566" s="2">
         <v>19</v>
@@ -21927,19 +21927,19 @@
     </row>
     <row r="567">
       <c r="A567" s="2">
-        <v>6813</v>
+        <v>7048</v>
       </c>
       <c r="B567" s="2" t="str">
-        <v>Torriani</v>
+        <v>De Marzi</v>
       </c>
       <c r="C567" s="2" t="str">
         <v/>
       </c>
       <c r="D567" s="2" t="str">
-        <v>Milan</v>
+        <v>Roma</v>
       </c>
       <c r="E567" s="2">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F567" s="2" t="str">
         <v>P</v>
@@ -21965,19 +21965,19 @@
     </row>
     <row r="568">
       <c r="A568" s="2">
-        <v>6682</v>
+        <v>6813</v>
       </c>
       <c r="B568" s="2" t="str">
-        <v>Pizzignacco</v>
+        <v>Torriani</v>
       </c>
       <c r="C568" s="2" t="str">
-        <v>*</v>
+        <v/>
       </c>
       <c r="D568" s="2" t="str">
-        <v>Monza</v>
+        <v>Milan</v>
       </c>
       <c r="E568" s="2">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F568" s="2" t="str">
         <v>P</v>
@@ -21986,13 +21986,13 @@
         <v>Por</v>
       </c>
       <c r="H568" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I568" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J568" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K568" s="2">
         <v>1</v>
@@ -22003,19 +22003,19 @@
     </row>
     <row r="569">
       <c r="A569" s="2">
-        <v>6671</v>
+        <v>6682</v>
       </c>
       <c r="B569" s="2" t="str">
-        <v>Grandi</v>
+        <v>Pizzignacco</v>
       </c>
       <c r="C569" s="2" t="str">
-        <v/>
+        <v>*</v>
       </c>
       <c r="D569" s="2" t="str">
-        <v>Venezia</v>
+        <v>Monza</v>
       </c>
       <c r="E569" s="2">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="F569" s="2" t="str">
         <v>P</v>
@@ -22024,13 +22024,13 @@
         <v>Por</v>
       </c>
       <c r="H569" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I569" s="2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J569" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K569" s="2">
         <v>1</v>
@@ -22041,19 +22041,19 @@
     </row>
     <row r="570">
       <c r="A570" s="2">
-        <v>6650</v>
+        <v>6671</v>
       </c>
       <c r="B570" s="2" t="str">
-        <v>Sherri</v>
+        <v>Grandi</v>
       </c>
       <c r="C570" s="2" t="str">
         <v/>
       </c>
       <c r="D570" s="2" t="str">
-        <v>Cagliari</v>
+        <v>Venezia</v>
       </c>
       <c r="E570" s="2">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F570" s="2" t="str">
         <v>P</v>
@@ -22079,19 +22079,19 @@
     </row>
     <row r="571">
       <c r="A571" s="2">
-        <v>6569</v>
+        <v>6650</v>
       </c>
       <c r="B571" s="2" t="str">
-        <v>Stolz</v>
+        <v>Sherri</v>
       </c>
       <c r="C571" s="2" t="str">
         <v/>
       </c>
       <c r="D571" s="2" t="str">
-        <v>Genoa</v>
+        <v>Cagliari</v>
       </c>
       <c r="E571" s="2">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F571" s="2" t="str">
         <v>P</v>
@@ -22117,19 +22117,19 @@
     </row>
     <row r="572">
       <c r="A572" s="2">
-        <v>6523</v>
+        <v>6569</v>
       </c>
       <c r="B572" s="2" t="str">
-        <v>Samooja</v>
+        <v>Stolz</v>
       </c>
       <c r="C572" s="2" t="str">
-        <v>*</v>
+        <v/>
       </c>
       <c r="D572" s="2" t="str">
-        <v>Lecce</v>
+        <v>Genoa</v>
       </c>
       <c r="E572" s="2">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F572" s="2" t="str">
         <v>P</v>
@@ -22155,19 +22155,19 @@
     </row>
     <row r="573">
       <c r="A573" s="2">
-        <v>6403</v>
+        <v>6523</v>
       </c>
       <c r="B573" s="2" t="str">
-        <v>Christensen O.</v>
+        <v>Samooja</v>
       </c>
       <c r="C573" s="2" t="str">
-        <v/>
+        <v>*</v>
       </c>
       <c r="D573" s="2" t="str">
-        <v>Fiorentina</v>
+        <v>Lecce</v>
       </c>
       <c r="E573" s="2">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F573" s="2" t="str">
         <v>P</v>
@@ -22193,19 +22193,19 @@
     </row>
     <row r="574">
       <c r="A574" s="2">
-        <v>5707</v>
+        <v>6403</v>
       </c>
       <c r="B574" s="2" t="str">
-        <v>Piana</v>
+        <v>Christensen O.</v>
       </c>
       <c r="C574" s="2" t="str">
         <v/>
       </c>
       <c r="D574" s="2" t="str">
-        <v>Udinese</v>
+        <v>Fiorentina</v>
       </c>
       <c r="E574" s="2">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F574" s="2" t="str">
         <v>P</v>
@@ -22231,19 +22231,19 @@
     </row>
     <row r="575">
       <c r="A575" s="2">
-        <v>5320</v>
+        <v>5707</v>
       </c>
       <c r="B575" s="2" t="str">
-        <v>Paleari</v>
+        <v>Piana</v>
       </c>
       <c r="C575" s="2" t="str">
         <v>*</v>
       </c>
       <c r="D575" s="2" t="str">
-        <v>Torino</v>
+        <v>Udinese</v>
       </c>
       <c r="E575" s="2">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="F575" s="2" t="str">
         <v>P</v>
@@ -22269,19 +22269,19 @@
     </row>
     <row r="576">
       <c r="A576" s="2">
-        <v>4957</v>
+        <v>5320</v>
       </c>
       <c r="B576" s="2" t="str">
-        <v>Montipò</v>
+        <v>Paleari</v>
       </c>
       <c r="C576" s="2" t="str">
-        <v/>
+        <v>*</v>
       </c>
       <c r="D576" s="2" t="str">
-        <v>Venezia</v>
+        <v>Torino</v>
       </c>
       <c r="E576" s="2">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F576" s="2" t="str">
         <v>P</v>
@@ -22307,19 +22307,19 @@
     </row>
     <row r="577">
       <c r="A577" s="2">
-        <v>4929</v>
+        <v>4957</v>
       </c>
       <c r="B577" s="2" t="str">
-        <v>Ciocci</v>
+        <v>Montipò</v>
       </c>
       <c r="C577" s="2" t="str">
-        <v>*</v>
+        <v/>
       </c>
       <c r="D577" s="2" t="str">
-        <v>Cagliari</v>
+        <v>Venezia</v>
       </c>
       <c r="E577" s="2">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F577" s="2" t="str">
         <v>P</v>
@@ -22345,19 +22345,19 @@
     </row>
     <row r="578">
       <c r="A578" s="2">
-        <v>4867</v>
+        <v>4929</v>
       </c>
       <c r="B578" s="2" t="str">
-        <v>Turati</v>
+        <v>Ciocci</v>
       </c>
       <c r="C578" s="2" t="str">
-        <v/>
+        <v>*</v>
       </c>
       <c r="D578" s="2" t="str">
-        <v>Sassuolo</v>
+        <v>Cagliari</v>
       </c>
       <c r="E578" s="2">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F578" s="2" t="str">
         <v>P</v>
@@ -22383,10 +22383,10 @@
     </row>
     <row r="579">
       <c r="A579" s="2">
-        <v>4518</v>
+        <v>4867</v>
       </c>
       <c r="B579" s="2" t="str">
-        <v>Russo A.</v>
+        <v>Turati</v>
       </c>
       <c r="C579" s="2" t="str">
         <v/>
@@ -22421,19 +22421,19 @@
     </row>
     <row r="580">
       <c r="A580" s="2">
-        <v>4468</v>
+        <v>4518</v>
       </c>
       <c r="B580" s="2" t="str">
-        <v>Bleve</v>
+        <v>Russo A.</v>
       </c>
       <c r="C580" s="2" t="str">
         <v/>
       </c>
       <c r="D580" s="2" t="str">
-        <v>Lecce</v>
+        <v>Sassuolo</v>
       </c>
       <c r="E580" s="2">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F580" s="2" t="str">
         <v>P</v>
@@ -22459,19 +22459,19 @@
     </row>
     <row r="581">
       <c r="A581" s="2">
-        <v>2874</v>
+        <v>4468</v>
       </c>
       <c r="B581" s="2" t="str">
-        <v>Ghidotti</v>
+        <v>Bleve</v>
       </c>
       <c r="C581" s="2" t="str">
         <v/>
       </c>
       <c r="D581" s="2" t="str">
-        <v>Parma</v>
+        <v>Lecce</v>
       </c>
       <c r="E581" s="2">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F581" s="2" t="str">
         <v>P</v>
@@ -22497,19 +22497,19 @@
     </row>
     <row r="582">
       <c r="A582" s="2">
-        <v>2845</v>
+        <v>2874</v>
       </c>
       <c r="B582" s="2" t="str">
-        <v>Contini</v>
+        <v>Ghidotti</v>
       </c>
       <c r="C582" s="2" t="str">
         <v/>
       </c>
       <c r="D582" s="2" t="str">
-        <v>Napoli</v>
+        <v>Parma</v>
       </c>
       <c r="E582" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F582" s="2" t="str">
         <v>P</v>
@@ -22535,19 +22535,19 @@
     </row>
     <row r="583">
       <c r="A583" s="2">
-        <v>2815</v>
+        <v>2845</v>
       </c>
       <c r="B583" s="2" t="str">
-        <v>Terracciano</v>
+        <v>Contini</v>
       </c>
       <c r="C583" s="2" t="str">
         <v/>
       </c>
       <c r="D583" s="2" t="str">
-        <v>Milan</v>
+        <v>Napoli</v>
       </c>
       <c r="E583" s="2">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F583" s="2" t="str">
         <v>P</v>
@@ -22573,16 +22573,16 @@
     </row>
     <row r="584">
       <c r="A584" s="2">
-        <v>2809</v>
+        <v>2815</v>
       </c>
       <c r="B584" s="2" t="str">
-        <v>Vigorito</v>
+        <v>Terracciano</v>
       </c>
       <c r="C584" s="2" t="str">
         <v/>
       </c>
       <c r="D584" s="2" t="str">
-        <v>Como</v>
+        <v>Milan</v>
       </c>
       <c r="E584" s="2">
         <v>36</v>
@@ -22611,19 +22611,19 @@
     </row>
     <row r="585">
       <c r="A585" s="2">
-        <v>2401</v>
+        <v>2809</v>
       </c>
       <c r="B585" s="2" t="str">
-        <v>Fruchtl</v>
+        <v>Vigorito</v>
       </c>
       <c r="C585" s="2" t="str">
-        <v>*</v>
+        <v/>
       </c>
       <c r="D585" s="2" t="str">
-        <v>Lecce</v>
+        <v>Como</v>
       </c>
       <c r="E585" s="2">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="F585" s="2" t="str">
         <v>P</v>
@@ -22649,19 +22649,19 @@
     </row>
     <row r="586">
       <c r="A586" s="2">
-        <v>2297</v>
+        <v>2401</v>
       </c>
       <c r="B586" s="2" t="str">
-        <v>Rossi F.</v>
+        <v>Fruchtl</v>
       </c>
       <c r="C586" s="2" t="str">
         <v>*</v>
       </c>
       <c r="D586" s="2" t="str">
-        <v>Atalanta</v>
+        <v>Lecce</v>
       </c>
       <c r="E586" s="2">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="F586" s="2" t="str">
         <v>P</v>
@@ -22687,19 +22687,19 @@
     </row>
     <row r="587">
       <c r="A587" s="2">
-        <v>2127</v>
+        <v>2297</v>
       </c>
       <c r="B587" s="2" t="str">
-        <v>Satalino</v>
+        <v>Rossi F.</v>
       </c>
       <c r="C587" s="2" t="str">
-        <v/>
+        <v>*</v>
       </c>
       <c r="D587" s="2" t="str">
-        <v>Sassuolo</v>
+        <v>Atalanta</v>
       </c>
       <c r="E587" s="2">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="F587" s="2" t="str">
         <v>P</v>
@@ -22725,19 +22725,19 @@
     </row>
     <row r="588">
       <c r="A588" s="2">
-        <v>1930</v>
+        <v>2127</v>
       </c>
       <c r="B588" s="2" t="str">
-        <v>Pinsoglio</v>
+        <v>Satalino</v>
       </c>
       <c r="C588" s="2" t="str">
         <v/>
       </c>
       <c r="D588" s="2" t="str">
-        <v>Juventus</v>
+        <v>Sassuolo</v>
       </c>
       <c r="E588" s="2">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="F588" s="2" t="str">
         <v>P</v>
@@ -22763,19 +22763,19 @@
     </row>
     <row r="589">
       <c r="A589" s="2">
-        <v>1926</v>
+        <v>1930</v>
       </c>
       <c r="B589" s="2" t="str">
-        <v>Di Gennaro</v>
+        <v>Pinsoglio</v>
       </c>
       <c r="C589" s="2" t="str">
         <v/>
       </c>
       <c r="D589" s="2" t="str">
-        <v>Inter</v>
+        <v>Juventus</v>
       </c>
       <c r="E589" s="2">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F589" s="2" t="str">
         <v>P</v>
@@ -22801,19 +22801,19 @@
     </row>
     <row r="590">
       <c r="A590" s="2">
-        <v>610</v>
+        <v>1926</v>
       </c>
       <c r="B590" s="2" t="str">
-        <v>Gollini</v>
+        <v>Di Gennaro</v>
       </c>
       <c r="C590" s="2" t="str">
         <v/>
       </c>
       <c r="D590" s="2" t="str">
-        <v>Roma</v>
+        <v>Inter</v>
       </c>
       <c r="E590" s="2">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F590" s="2" t="str">
         <v>P</v>
@@ -22839,19 +22839,19 @@
     </row>
     <row r="591">
       <c r="A591" s="2">
-        <v>543</v>
+        <v>610</v>
       </c>
       <c r="B591" s="2" t="str">
-        <v>Padelli</v>
+        <v>Gollini</v>
       </c>
       <c r="C591" s="2" t="str">
         <v/>
       </c>
       <c r="D591" s="2" t="str">
-        <v>Udinese</v>
+        <v>Roma</v>
       </c>
       <c r="E591" s="2">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F591" s="2" t="str">
         <v>P</v>
@@ -22877,19 +22877,19 @@
     </row>
     <row r="592">
       <c r="A592" s="2">
-        <v>219</v>
+        <v>543</v>
       </c>
       <c r="B592" s="2" t="str">
-        <v>Sommariva</v>
+        <v>Padelli</v>
       </c>
       <c r="C592" s="2" t="str">
         <v/>
       </c>
       <c r="D592" s="2" t="str">
-        <v>Genoa</v>
+        <v>Udinese</v>
       </c>
       <c r="E592" s="2">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="F592" s="2" t="str">
         <v>P</v>
@@ -22915,19 +22915,19 @@
     </row>
     <row r="593">
       <c r="A593" s="2">
-        <v>158</v>
+        <v>219</v>
       </c>
       <c r="B593" s="2" t="str">
-        <v>Lezzerini</v>
+        <v>Sommariva</v>
       </c>
       <c r="C593" s="2" t="str">
         <v/>
       </c>
       <c r="D593" s="2" t="str">
-        <v>Fiorentina</v>
+        <v>Genoa</v>
       </c>
       <c r="E593" s="2">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F593" s="2" t="str">
         <v>P</v>
@@ -22953,19 +22953,19 @@
     </row>
     <row r="594">
       <c r="A594" s="2">
-        <v>4</v>
+        <v>158</v>
       </c>
       <c r="B594" s="2" t="str">
-        <v>Sportiello</v>
+        <v>Lezzerini</v>
       </c>
       <c r="C594" s="2" t="str">
         <v/>
       </c>
       <c r="D594" s="2" t="str">
-        <v>Atalanta</v>
+        <v>Fiorentina</v>
       </c>
       <c r="E594" s="2">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F594" s="2" t="str">
         <v>P</v>
@@ -22991,19 +22991,19 @@
     </row>
     <row r="595">
       <c r="A595" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B595" s="2" t="str">
-        <v>Radunovic</v>
+        <v>Sportiello</v>
       </c>
       <c r="C595" s="2" t="str">
         <v/>
       </c>
       <c r="D595" s="2" t="str">
-        <v>Cagliari</v>
+        <v>Atalanta</v>
       </c>
       <c r="E595" s="2">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F595" s="2" t="str">
         <v>P</v>
@@ -23027,9 +23027,47 @@
         <v>1</v>
       </c>
     </row>
+    <row r="596">
+      <c r="A596" s="2">
+        <v>3</v>
+      </c>
+      <c r="B596" s="2" t="str">
+        <v>Radunovic</v>
+      </c>
+      <c r="C596" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D596" s="2" t="str">
+        <v>Cagliari</v>
+      </c>
+      <c r="E596" s="2">
+        <v>30</v>
+      </c>
+      <c r="F596" s="2" t="str">
+        <v>P</v>
+      </c>
+      <c r="G596" s="2" t="str">
+        <v>Por</v>
+      </c>
+      <c r="H596" s="2">
+        <v>0</v>
+      </c>
+      <c r="I596" s="2">
+        <v>0</v>
+      </c>
+      <c r="J596" s="2">
+        <v>0</v>
+      </c>
+      <c r="K596" s="2">
+        <v>1</v>
+      </c>
+      <c r="L596" s="2">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N595"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N596"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>